<commit_message>
Pedidos ePan com EAN confirmado do catálogo Panpharma
- Coluna EAN dos 2 pedidos substituída pelo EAN do painel ePan PRO 10/09
  (conta 712093), casado pelo código Panpharma ("EAN ePan (confirmado)").
- 331 itens já coincidiam com o EAN interno; 7 substituídos (DUN-14 e
  códigos de embalagem alternativa); nenhum item sem EAN no catálogo.
- Verificação de preços regerada; script de verificação aceita o novo
  nome de coluna.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VLivvbyTHZf5HaiMxTfGPo
</commit_message>
<xml_diff>
--- a/cotacoes/2026-09-08/fechamento/PEDIDO_EPAN_DEMAIS_10-09-2026.xlsx
+++ b/cotacoes/2026-09-08/fechamento/PEDIDO_EPAN_DEMAIS_10-09-2026.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>EAN</t>
+          <t>EAN ePan (confirmado)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>0000042277217</t>
+          <t>42277217</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>7891000319598</t>
+          <t>7891000319581</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -9283,7 +9283,7 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>7891000062739</t>
+          <t>7891000062722</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>47896512900058</t>
+          <t>7896512900050</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>37896512912306</t>
+          <t>7896512900166</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -16411,6 +16411,7 @@
         <v/>
       </c>
     </row>
+    <row r="236"/>
     <row r="237">
       <c r="A237" s="9" t="inlineStr">
         <is>

</xml_diff>